<commit_message>
Weekly plan template: one tab per brand (CFBL Practice, Institute, MUSA)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019WVVTo5U2894eKUuHPjTGE
</commit_message>
<xml_diff>
--- a/marketing/templates/CFBL_Weekly_Plan_TEMPLATE.xlsx
+++ b/marketing/templates/CFBL_Weekly_Plan_TEMPLATE.xlsx
@@ -7,8 +7,10 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Weekly Plan" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="How to Use" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="CFBL — Practice" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="CFBL Institute" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="MUSA" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="How to Use" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -27,9 +29,23 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="007A7A7A"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00F0EAE0"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00F1E8D8"/>
       <sz val="11"/>
     </font>
     <font>
@@ -46,7 +62,7 @@
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -61,6 +77,26 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00F5F1EA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="003D5A52"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EFF3EE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="006E1F23"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F6EFE3"/>
       </patternFill>
     </fill>
   </fills>
@@ -90,7 +126,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -101,13 +137,26 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -475,20 +524,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K8"/>
+  <dimension ref="A1:J11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="40" customWidth="1" min="7" max="7"/>
-    <col width="40" customWidth="1" min="8" max="8"/>
-    <col width="28" customWidth="1" min="9" max="9"/>
-    <col width="30" customWidth="1" min="10" max="10"/>
-    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="42" customWidth="1" min="6" max="6"/>
+    <col width="42" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="8" max="8"/>
+    <col width="30" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -509,319 +557,222 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>BRAND</t>
+          <t>FORMAT</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>FORMAT</t>
+          <t>CONTENT TYPE</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>CONTENT TYPE</t>
+          <t>POST TOPIC</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>POST TOPIC</t>
+          <t>BUSINESS OBJECTIVE</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>BUSINESS OBJECTIVE</t>
+          <t>CTA</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>CTA</t>
+          <t>LINK</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>LINK</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
           <t>STATUS</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="54" customHeight="1">
-      <c r="A2" s="2" t="inlineStr"/>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Mon</t>
-        </is>
-      </c>
+    <row r="2" ht="48" customHeight="1">
+      <c r="A2" s="2" t="n"/>
+      <c r="B2" s="2" t="n"/>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Dr. Niki</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>CFBL Institute</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Carousel</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>Educational</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr"/>
-      <c r="H2" s="2" t="inlineStr"/>
-      <c r="I2" s="2" t="inlineStr"/>
-      <c r="J2" s="2" t="inlineStr"/>
-      <c r="K2" s="2" t="inlineStr">
-        <is>
-          <t>Plan</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="54" customHeight="1">
-      <c r="A3" s="3" t="inlineStr"/>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>Tue</t>
-        </is>
-      </c>
+          <t>CFBL</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="n"/>
+      <c r="E2" s="2" t="n"/>
+      <c r="F2" s="2" t="n"/>
+      <c r="G2" s="2" t="n"/>
+      <c r="H2" s="2" t="n"/>
+      <c r="I2" s="2" t="n"/>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Plan</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="48" customHeight="1">
+      <c r="A3" s="3" t="n"/>
+      <c r="B3" s="3" t="n"/>
       <c r="C3" s="3" t="inlineStr">
         <is>
           <t>CFBL</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>Center for Balanced Living</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>Carousel</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>Educational</t>
-        </is>
-      </c>
-      <c r="G3" s="3" t="inlineStr"/>
-      <c r="H3" s="3" t="inlineStr"/>
-      <c r="I3" s="3" t="inlineStr"/>
-      <c r="J3" s="3" t="inlineStr"/>
-      <c r="K3" s="3" t="inlineStr">
-        <is>
-          <t>Plan</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="54" customHeight="1">
-      <c r="A4" s="2" t="inlineStr"/>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>Wed</t>
-        </is>
-      </c>
+      <c r="D3" s="3" t="n"/>
+      <c r="E3" s="3" t="n"/>
+      <c r="F3" s="3" t="n"/>
+      <c r="G3" s="3" t="n"/>
+      <c r="H3" s="3" t="n"/>
+      <c r="I3" s="3" t="n"/>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>Plan</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="48" customHeight="1">
+      <c r="A4" s="2" t="n"/>
+      <c r="B4" s="2" t="n"/>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Dr. Niki</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>CFBL Institute</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>Single image</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>Promotional</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr"/>
-      <c r="H4" s="2" t="inlineStr"/>
-      <c r="I4" s="2" t="inlineStr"/>
-      <c r="J4" s="2" t="inlineStr"/>
-      <c r="K4" s="2" t="inlineStr">
-        <is>
-          <t>Plan</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="54" customHeight="1">
-      <c r="A5" s="3" t="inlineStr"/>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>Thu</t>
-        </is>
-      </c>
+          <t>CFBL</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="n"/>
+      <c r="E4" s="2" t="n"/>
+      <c r="F4" s="2" t="n"/>
+      <c r="G4" s="2" t="n"/>
+      <c r="H4" s="2" t="n"/>
+      <c r="I4" s="2" t="n"/>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>Plan</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="48" customHeight="1">
+      <c r="A5" s="3" t="n"/>
+      <c r="B5" s="3" t="n"/>
       <c r="C5" s="3" t="inlineStr">
         <is>
           <t>CFBL</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>Center for Balanced Living</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="inlineStr">
-        <is>
-          <t>Single image</t>
-        </is>
-      </c>
-      <c r="F5" s="3" t="inlineStr">
-        <is>
-          <t>Community</t>
-        </is>
-      </c>
-      <c r="G5" s="3" t="inlineStr"/>
-      <c r="H5" s="3" t="inlineStr"/>
-      <c r="I5" s="3" t="inlineStr"/>
-      <c r="J5" s="3" t="inlineStr"/>
-      <c r="K5" s="3" t="inlineStr">
-        <is>
-          <t>Plan</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="54" customHeight="1">
-      <c r="A6" s="2" t="inlineStr"/>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>Fri</t>
-        </is>
-      </c>
+      <c r="D5" s="3" t="n"/>
+      <c r="E5" s="3" t="n"/>
+      <c r="F5" s="3" t="n"/>
+      <c r="G5" s="3" t="n"/>
+      <c r="H5" s="3" t="n"/>
+      <c r="I5" s="3" t="n"/>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>Plan</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="48" customHeight="1">
+      <c r="A6" s="2" t="n"/>
+      <c r="B6" s="2" t="n"/>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Dr. Niki</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>CFBL Institute</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>Reel</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>Educational</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr"/>
-      <c r="H6" s="2" t="inlineStr"/>
-      <c r="I6" s="2" t="inlineStr"/>
-      <c r="J6" s="2" t="inlineStr"/>
-      <c r="K6" s="2" t="inlineStr">
-        <is>
-          <t>Plan</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="54" customHeight="1">
-      <c r="A7" s="3" t="inlineStr"/>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>Sat</t>
-        </is>
-      </c>
+          <t>CFBL</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="n"/>
+      <c r="E6" s="2" t="n"/>
+      <c r="F6" s="2" t="n"/>
+      <c r="G6" s="2" t="n"/>
+      <c r="H6" s="2" t="n"/>
+      <c r="I6" s="2" t="n"/>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>Plan</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="48" customHeight="1">
+      <c r="A7" s="3" t="n"/>
+      <c r="B7" s="3" t="n"/>
       <c r="C7" s="3" t="inlineStr">
         <is>
           <t>CFBL</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>Center for Balanced Living</t>
-        </is>
-      </c>
-      <c r="E7" s="3" t="inlineStr">
-        <is>
-          <t>Single image</t>
-        </is>
-      </c>
-      <c r="F7" s="3" t="inlineStr">
-        <is>
-          <t>Community</t>
-        </is>
-      </c>
-      <c r="G7" s="3" t="inlineStr"/>
-      <c r="H7" s="3" t="inlineStr"/>
-      <c r="I7" s="3" t="inlineStr"/>
-      <c r="J7" s="3" t="inlineStr"/>
-      <c r="K7" s="3" t="inlineStr">
-        <is>
-          <t>Plan</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="54" customHeight="1">
-      <c r="A8" s="2" t="inlineStr"/>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>Sun</t>
-        </is>
-      </c>
+      <c r="D7" s="3" t="n"/>
+      <c r="E7" s="3" t="n"/>
+      <c r="F7" s="3" t="n"/>
+      <c r="G7" s="3" t="n"/>
+      <c r="H7" s="3" t="n"/>
+      <c r="I7" s="3" t="n"/>
+      <c r="J7" s="3" t="inlineStr">
+        <is>
+          <t>Plan</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="48" customHeight="1">
+      <c r="A8" s="2" t="n"/>
+      <c r="B8" s="2" t="n"/>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Dr. Niki</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>CFBL Institute</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>Carousel</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>Promotional</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="inlineStr"/>
-      <c r="H8" s="2" t="inlineStr"/>
-      <c r="I8" s="2" t="inlineStr"/>
-      <c r="J8" s="2" t="inlineStr"/>
-      <c r="K8" s="2" t="inlineStr">
-        <is>
-          <t>Plan</t>
+          <t>CFBL</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="n"/>
+      <c r="E8" s="2" t="n"/>
+      <c r="F8" s="2" t="n"/>
+      <c r="G8" s="2" t="n"/>
+      <c r="H8" s="2" t="n"/>
+      <c r="I8" s="2" t="n"/>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>Plan</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="48" customHeight="1">
+      <c r="A9" s="3" t="n"/>
+      <c r="B9" s="3" t="n"/>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>CFBL</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="n"/>
+      <c r="E9" s="3" t="n"/>
+      <c r="F9" s="3" t="n"/>
+      <c r="G9" s="3" t="n"/>
+      <c r="H9" s="3" t="n"/>
+      <c r="I9" s="3" t="n"/>
+      <c r="J9" s="3" t="inlineStr">
+        <is>
+          <t>Plan</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Weekly mix across all 3 brands: aim 3 Educational · 2 Community · 2 Promotional.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <dataValidations count="5">
+    <dataValidation sqref="B2:B30" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Mon,Tue,Wed,Thu,Fri,Sat,Sun"</formula1>
+    </dataValidation>
     <dataValidation sqref="C2:C30" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"CFBL,Dr. Niki"</formula1>
     </dataValidation>
     <dataValidation sqref="D2:D30" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Center for Balanced Living,CFBL Institute,MUSA"</formula1>
+      <formula1>"Carousel,Single image,Reel,Story"</formula1>
     </dataValidation>
     <dataValidation sqref="E2:E30" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Carousel,Single image,Reel,Story"</formula1>
-    </dataValidation>
-    <dataValidation sqref="F2:F30" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Educational,Community,Promotional"</formula1>
     </dataValidation>
-    <dataValidation sqref="K2:K30" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J2:J30" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Plan,Copy done,Design done,Ready for CSV,Scheduled"</formula1>
     </dataValidation>
   </dataValidations>
@@ -835,137 +786,654 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A20"/>
+  <dimension ref="A1:J11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="42" customWidth="1" min="6" max="6"/>
+    <col width="42" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="8" max="8"/>
+    <col width="30" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>DATE</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>DAY</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>PAGE</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>FORMAT</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>CONTENT TYPE</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="inlineStr">
+        <is>
+          <t>POST TOPIC</t>
+        </is>
+      </c>
+      <c r="G1" s="5" t="inlineStr">
+        <is>
+          <t>BUSINESS OBJECTIVE</t>
+        </is>
+      </c>
+      <c r="H1" s="5" t="inlineStr">
+        <is>
+          <t>CTA</t>
+        </is>
+      </c>
+      <c r="I1" s="5" t="inlineStr">
+        <is>
+          <t>LINK</t>
+        </is>
+      </c>
+      <c r="J1" s="5" t="inlineStr">
+        <is>
+          <t>STATUS</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="48" customHeight="1">
+      <c r="A2" s="6" t="n"/>
+      <c r="B2" s="6" t="n"/>
+      <c r="C2" s="6" t="inlineStr">
+        <is>
+          <t>Dr. Niki</t>
+        </is>
+      </c>
+      <c r="D2" s="6" t="n"/>
+      <c r="E2" s="6" t="n"/>
+      <c r="F2" s="6" t="n"/>
+      <c r="G2" s="6" t="n"/>
+      <c r="H2" s="6" t="n"/>
+      <c r="I2" s="6" t="n"/>
+      <c r="J2" s="6" t="inlineStr">
+        <is>
+          <t>Plan</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="48" customHeight="1">
+      <c r="A3" s="3" t="n"/>
+      <c r="B3" s="3" t="n"/>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Dr. Niki</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="n"/>
+      <c r="E3" s="3" t="n"/>
+      <c r="F3" s="3" t="n"/>
+      <c r="G3" s="3" t="n"/>
+      <c r="H3" s="3" t="n"/>
+      <c r="I3" s="3" t="n"/>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>Plan</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="48" customHeight="1">
+      <c r="A4" s="6" t="n"/>
+      <c r="B4" s="6" t="n"/>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>Dr. Niki</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="n"/>
+      <c r="E4" s="6" t="n"/>
+      <c r="F4" s="6" t="n"/>
+      <c r="G4" s="6" t="n"/>
+      <c r="H4" s="6" t="n"/>
+      <c r="I4" s="6" t="n"/>
+      <c r="J4" s="6" t="inlineStr">
+        <is>
+          <t>Plan</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="48" customHeight="1">
+      <c r="A5" s="3" t="n"/>
+      <c r="B5" s="3" t="n"/>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Dr. Niki</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="n"/>
+      <c r="E5" s="3" t="n"/>
+      <c r="F5" s="3" t="n"/>
+      <c r="G5" s="3" t="n"/>
+      <c r="H5" s="3" t="n"/>
+      <c r="I5" s="3" t="n"/>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>Plan</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="48" customHeight="1">
+      <c r="A6" s="6" t="n"/>
+      <c r="B6" s="6" t="n"/>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>Dr. Niki</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="n"/>
+      <c r="E6" s="6" t="n"/>
+      <c r="F6" s="6" t="n"/>
+      <c r="G6" s="6" t="n"/>
+      <c r="H6" s="6" t="n"/>
+      <c r="I6" s="6" t="n"/>
+      <c r="J6" s="6" t="inlineStr">
+        <is>
+          <t>Plan</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="48" customHeight="1">
+      <c r="A7" s="3" t="n"/>
+      <c r="B7" s="3" t="n"/>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Dr. Niki</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="n"/>
+      <c r="E7" s="3" t="n"/>
+      <c r="F7" s="3" t="n"/>
+      <c r="G7" s="3" t="n"/>
+      <c r="H7" s="3" t="n"/>
+      <c r="I7" s="3" t="n"/>
+      <c r="J7" s="3" t="inlineStr">
+        <is>
+          <t>Plan</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="48" customHeight="1">
+      <c r="A8" s="6" t="n"/>
+      <c r="B8" s="6" t="n"/>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>Dr. Niki</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="n"/>
+      <c r="E8" s="6" t="n"/>
+      <c r="F8" s="6" t="n"/>
+      <c r="G8" s="6" t="n"/>
+      <c r="H8" s="6" t="n"/>
+      <c r="I8" s="6" t="n"/>
+      <c r="J8" s="6" t="inlineStr">
+        <is>
+          <t>Plan</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="48" customHeight="1">
+      <c r="A9" s="3" t="n"/>
+      <c r="B9" s="3" t="n"/>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Dr. Niki</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="n"/>
+      <c r="E9" s="3" t="n"/>
+      <c r="F9" s="3" t="n"/>
+      <c r="G9" s="3" t="n"/>
+      <c r="H9" s="3" t="n"/>
+      <c r="I9" s="3" t="n"/>
+      <c r="J9" s="3" t="inlineStr">
+        <is>
+          <t>Plan</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Weekly mix across all 3 brands: aim 3 Educational · 2 Community · 2 Promotional.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="5">
+    <dataValidation sqref="B2:B30" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Mon,Tue,Wed,Thu,Fri,Sat,Sun"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C2:C30" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"CFBL,Dr. Niki"</formula1>
+    </dataValidation>
+    <dataValidation sqref="D2:D30" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Carousel,Single image,Reel,Story"</formula1>
+    </dataValidation>
+    <dataValidation sqref="E2:E30" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Educational,Community,Promotional"</formula1>
+    </dataValidation>
+    <dataValidation sqref="J2:J30" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Plan,Copy done,Design done,Ready for CSV,Scheduled"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="42" customWidth="1" min="6" max="6"/>
+    <col width="42" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="8" max="8"/>
+    <col width="30" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>DATE</t>
+        </is>
+      </c>
+      <c r="B1" s="7" t="inlineStr">
+        <is>
+          <t>DAY</t>
+        </is>
+      </c>
+      <c r="C1" s="7" t="inlineStr">
+        <is>
+          <t>PAGE</t>
+        </is>
+      </c>
+      <c r="D1" s="7" t="inlineStr">
+        <is>
+          <t>FORMAT</t>
+        </is>
+      </c>
+      <c r="E1" s="7" t="inlineStr">
+        <is>
+          <t>CONTENT TYPE</t>
+        </is>
+      </c>
+      <c r="F1" s="7" t="inlineStr">
+        <is>
+          <t>POST TOPIC</t>
+        </is>
+      </c>
+      <c r="G1" s="7" t="inlineStr">
+        <is>
+          <t>BUSINESS OBJECTIVE</t>
+        </is>
+      </c>
+      <c r="H1" s="7" t="inlineStr">
+        <is>
+          <t>CTA</t>
+        </is>
+      </c>
+      <c r="I1" s="7" t="inlineStr">
+        <is>
+          <t>LINK</t>
+        </is>
+      </c>
+      <c r="J1" s="7" t="inlineStr">
+        <is>
+          <t>STATUS</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="48" customHeight="1">
+      <c r="A2" s="8" t="n"/>
+      <c r="B2" s="8" t="n"/>
+      <c r="C2" s="8" t="inlineStr">
+        <is>
+          <t>Dr. Niki</t>
+        </is>
+      </c>
+      <c r="D2" s="8" t="n"/>
+      <c r="E2" s="8" t="n"/>
+      <c r="F2" s="8" t="n"/>
+      <c r="G2" s="8" t="n"/>
+      <c r="H2" s="8" t="n"/>
+      <c r="I2" s="8" t="n"/>
+      <c r="J2" s="8" t="inlineStr">
+        <is>
+          <t>Plan</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="48" customHeight="1">
+      <c r="A3" s="3" t="n"/>
+      <c r="B3" s="3" t="n"/>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Dr. Niki</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="n"/>
+      <c r="E3" s="3" t="n"/>
+      <c r="F3" s="3" t="n"/>
+      <c r="G3" s="3" t="n"/>
+      <c r="H3" s="3" t="n"/>
+      <c r="I3" s="3" t="n"/>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>Plan</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="48" customHeight="1">
+      <c r="A4" s="8" t="n"/>
+      <c r="B4" s="8" t="n"/>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>Dr. Niki</t>
+        </is>
+      </c>
+      <c r="D4" s="8" t="n"/>
+      <c r="E4" s="8" t="n"/>
+      <c r="F4" s="8" t="n"/>
+      <c r="G4" s="8" t="n"/>
+      <c r="H4" s="8" t="n"/>
+      <c r="I4" s="8" t="n"/>
+      <c r="J4" s="8" t="inlineStr">
+        <is>
+          <t>Plan</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="48" customHeight="1">
+      <c r="A5" s="3" t="n"/>
+      <c r="B5" s="3" t="n"/>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Dr. Niki</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="n"/>
+      <c r="E5" s="3" t="n"/>
+      <c r="F5" s="3" t="n"/>
+      <c r="G5" s="3" t="n"/>
+      <c r="H5" s="3" t="n"/>
+      <c r="I5" s="3" t="n"/>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>Plan</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="48" customHeight="1">
+      <c r="A6" s="8" t="n"/>
+      <c r="B6" s="8" t="n"/>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>Dr. Niki</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="n"/>
+      <c r="E6" s="8" t="n"/>
+      <c r="F6" s="8" t="n"/>
+      <c r="G6" s="8" t="n"/>
+      <c r="H6" s="8" t="n"/>
+      <c r="I6" s="8" t="n"/>
+      <c r="J6" s="8" t="inlineStr">
+        <is>
+          <t>Plan</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="48" customHeight="1">
+      <c r="A7" s="3" t="n"/>
+      <c r="B7" s="3" t="n"/>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Dr. Niki</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="n"/>
+      <c r="E7" s="3" t="n"/>
+      <c r="F7" s="3" t="n"/>
+      <c r="G7" s="3" t="n"/>
+      <c r="H7" s="3" t="n"/>
+      <c r="I7" s="3" t="n"/>
+      <c r="J7" s="3" t="inlineStr">
+        <is>
+          <t>Plan</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="48" customHeight="1">
+      <c r="A8" s="8" t="n"/>
+      <c r="B8" s="8" t="n"/>
+      <c r="C8" s="8" t="inlineStr">
+        <is>
+          <t>Dr. Niki</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="n"/>
+      <c r="E8" s="8" t="n"/>
+      <c r="F8" s="8" t="n"/>
+      <c r="G8" s="8" t="n"/>
+      <c r="H8" s="8" t="n"/>
+      <c r="I8" s="8" t="n"/>
+      <c r="J8" s="8" t="inlineStr">
+        <is>
+          <t>Plan</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="48" customHeight="1">
+      <c r="A9" s="3" t="n"/>
+      <c r="B9" s="3" t="n"/>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Dr. Niki</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="n"/>
+      <c r="E9" s="3" t="n"/>
+      <c r="F9" s="3" t="n"/>
+      <c r="G9" s="3" t="n"/>
+      <c r="H9" s="3" t="n"/>
+      <c r="I9" s="3" t="n"/>
+      <c r="J9" s="3" t="inlineStr">
+        <is>
+          <t>Plan</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Weekly mix across all 3 brands: aim 3 Educational · 2 Community · 2 Promotional.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="5">
+    <dataValidation sqref="B2:B30" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Mon,Tue,Wed,Thu,Fri,Sat,Sun"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C2:C30" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"CFBL,Dr. Niki"</formula1>
+    </dataValidation>
+    <dataValidation sqref="D2:D30" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Carousel,Single image,Reel,Story"</formula1>
+    </dataValidation>
+    <dataValidation sqref="E2:E30" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Educational,Community,Promotional"</formula1>
+    </dataValidation>
+    <dataValidation sqref="J2:J30" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Plan,Copy done,Design done,Ready for CSV,Scheduled"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
-        <is>
-          <t>CFBL Weekly Content System — How to Use This Plan</t>
+      <c r="A1" s="9" t="inlineStr">
+        <is>
+          <t>CFBL Weekly Content System — How to Use</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="inlineStr"/>
+      <c r="A2" s="10" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="inlineStr">
+      <c r="A3" s="10" t="inlineStr">
+        <is>
+          <t>ONE TAB PER BRAND. Plan each brand on its own tab; I merge all three into one Metricool bulk CSV at the end.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="10" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="11" t="inlineStr">
         <is>
           <t>THE WEEKLY LOOP</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="5" t="inlineStr">
-        <is>
-          <t>1. PLAN (Thu/Fri): fill one row per post below. Keep the mix: 3 Educational · 2 Community · 2 Promotional.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="5" t="inlineStr">
-        <is>
-          <t>2. COPY: paste the ChatGPT prompt (bottom) + your rows → get captions, hashtags, Google versions.</t>
-        </is>
-      </c>
-    </row>
     <row r="6">
-      <c r="A6" s="5" t="inlineStr">
-        <is>
-          <t>3. DESIGN (weekend): build in Canva templates (Gamma for the occasional educational carousel/newsletter); drop in real photos.</t>
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t>1. PLAN (Thu/Fri): fill rows on each brand tab. Across all brands, aim 3 Educational · 2 Community · 2 Promotional.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>4. ASSEMBLE (Mon): hand finished PNGs to Claude → get the Metricool bulk CSV.</t>
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t>2. COPY: paste the ChatGPT prompt (below) + your rows → captions, hashtags, Google versions.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="inlineStr">
+      <c r="A8" s="10" t="inlineStr">
+        <is>
+          <t>3. DESIGN (weekend): Canva templates (+ Gamma for occasional carousels/newsletter); drop in real photos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>4. ASSEMBLE (Mon): upload finished PNGs to Shopify Files → I read the URLs + build the Metricool bulk CSV.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="10" t="inlineStr">
         <is>
           <t>5. SCHEDULE: import CSV to Metricool → add IG Collab on CFBL posts + Google versions → schedule.</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="5" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="6" t="inlineStr">
-        <is>
-          <t>CONTENT MIX (why it builds community AND enrollment)</t>
-        </is>
-      </c>
-    </row>
     <row r="11">
-      <c r="A11" s="5" t="inlineStr">
-        <is>
-          <t>Educational = trust/authority. Community = connection/engagement. Promotional = soft enrollment. Aim 3/2/2 weekly.</t>
-        </is>
-      </c>
+      <c r="A11" s="10" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="5" t="inlineStr"/>
+      <c r="A12" s="11" t="inlineStr">
+        <is>
+          <t>BRAND → PAGE → LOOK</t>
+        </is>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="6" t="inlineStr">
-        <is>
-          <t>BRAND → PAGE → LOOK</t>
+      <c r="A13" s="10" t="inlineStr">
+        <is>
+          <t>CFBL — Practice (evaluations, therapy, groups, community) → CFBL page → navy/white → CFBL logo.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="5" t="inlineStr">
-        <is>
-          <t>Center for Balanced Living (practice: evaluations, therapy, groups, community) → CFBL page → navy/white → CFBL logo.</t>
+      <c r="A14" s="10" t="inlineStr">
+        <is>
+          <t>CFBL Institute (trainings/workshops) → Dr. Niki page → green/cream → CFBL Institute logo.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="5" t="inlineStr">
-        <is>
-          <t>CFBL Institute (trainings/workshops) → Dr. Niki page → green/cream → CFBL Institute logo.</t>
+      <c r="A15" s="10" t="inlineStr">
+        <is>
+          <t>MUSA (blog, essays, newsletter) → Dr. Niki page → gold/red → MUSA styling.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="5" t="inlineStr">
-        <is>
-          <t>MUSA (blog, essays, newsletter) → Dr. Niki page → gold/red → MUSA styling.</t>
+      <c r="A16" s="10" t="inlineStr">
+        <is>
+          <t>On CFBL-page Instagram posts, add Dr. Niki as a Collaborator.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="5" t="inlineStr">
-        <is>
-          <t>On CFBL-page Instagram posts, add Dr. Niki as a Collaborator.</t>
-        </is>
-      </c>
+      <c r="A17" s="10" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" s="5" t="inlineStr"/>
+      <c r="A18" s="11" t="inlineStr">
+        <is>
+          <t>REUSABLE CHATGPT / CLAUDE CAPTION PROMPT (copy below)</t>
+        </is>
+      </c>
     </row>
     <row r="19">
-      <c r="A19" s="6" t="inlineStr">
-        <is>
-          <t>REUSABLE CHATGPT / CLAUDE CAPTION PROMPT (copy everything below the line)</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="5" t="inlineStr">
+      <c r="A19" s="10" t="inlineStr">
         <is>
           <t>You are the social media copywriter for Center for Balanced Living (practice), CFBL Institute (clinician trainings), and MUSA (writing). Voice: warm, authentic, emotionally safe, professional. Educate and build trust — never clickbait, never manipulative, never invent dates/prices/credentials. Institute posts are peer-to-peer (clinicians); practice posts are warm and relational.
 For each row I give you (date, brand, format, topic, objective, CTA), write:
 1) A caption in that brand's voice (don't shorten educational content).
-2) 5–6 relevant hashtags (no invented trending tags) for the FIRST COMMENT.
-3) A short 1–2 sentence Google Business Profile version (no hashtags) + a CTA button label.
+2) 5-6 relevant hashtags (no invented trending tags) for the FIRST COMMENT.
+3) A short 1-2 sentence Google Business Profile version (no hashtags) + a CTA button label.
 Keep all facts exactly as I provide them. Ask me if anything required (fee, link, credential) is missing.
 Here is this week's plan:
 [paste your rows]</t>

</xml_diff>